<commit_message>
added data and notes from outplant check
</commit_message>
<xml_diff>
--- a/data/metadata/experiment_metadata.xlsx
+++ b/data/metadata/experiment_metadata.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashuffmyer/MyProjects/oysters/manchester-hardening/data/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4866CB6D-B8D4-F24A-B48C-4F797B42BC9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B5F8E3-CBAD-7847-A6C6-3094C615985C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15940" yWindow="760" windowWidth="14060" windowHeight="17600" xr2:uid="{910C5C9C-1199-2F4F-A6BD-E003E55895D4}"/>
+    <workbookView xWindow="50220" yWindow="-1100" windowWidth="14060" windowHeight="17600" xr2:uid="{910C5C9C-1199-2F4F-A6BD-E003E55895D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="25">
   <si>
     <t>tank</t>
   </si>
@@ -102,6 +102,15 @@
   </si>
   <si>
     <t>starting_oysters</t>
+  </si>
+  <si>
+    <t>20260107_split</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -473,13 +482,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026AE326-2012-A844-AB6A-692D667495E5}">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -498,8 +508,11 @@
       <c r="F1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>52</v>
       </c>
@@ -518,8 +531,11 @@
       <c r="F2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>56</v>
       </c>
@@ -538,8 +554,11 @@
       <c r="F3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>60</v>
       </c>
@@ -558,8 +577,11 @@
       <c r="F4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>62</v>
       </c>
@@ -578,8 +600,11 @@
       <c r="F5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>65</v>
       </c>
@@ -598,8 +623,11 @@
       <c r="F6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>73</v>
       </c>
@@ -618,8 +646,11 @@
       <c r="F7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>79</v>
       </c>
@@ -638,8 +669,11 @@
       <c r="F8" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>86</v>
       </c>
@@ -658,8 +692,11 @@
       <c r="F9" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>87</v>
       </c>
@@ -678,8 +715,11 @@
       <c r="F10" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>90</v>
       </c>
@@ -698,8 +738,11 @@
       <c r="F11" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>53</v>
       </c>
@@ -718,8 +761,11 @@
       <c r="F12" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>57</v>
       </c>
@@ -738,8 +784,11 @@
       <c r="F13" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>61</v>
       </c>
@@ -758,8 +807,11 @@
       <c r="F14" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>64</v>
       </c>
@@ -778,8 +830,11 @@
       <c r="F15" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>67</v>
       </c>
@@ -798,8 +853,11 @@
       <c r="F16" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>72</v>
       </c>
@@ -818,8 +876,11 @@
       <c r="F17" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>78</v>
       </c>
@@ -838,8 +899,11 @@
       <c r="F18" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>82</v>
       </c>
@@ -858,8 +922,11 @@
       <c r="F19" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>85</v>
       </c>
@@ -878,8 +945,11 @@
       <c r="F20" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>88</v>
       </c>
@@ -898,8 +968,11 @@
       <c r="F21" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>55</v>
       </c>
@@ -918,8 +991,11 @@
       <c r="F22" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>58</v>
       </c>
@@ -938,8 +1014,11 @@
       <c r="F23" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>66</v>
       </c>
@@ -958,8 +1037,11 @@
       <c r="F24" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>68</v>
       </c>
@@ -978,8 +1060,11 @@
       <c r="F25" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>70</v>
       </c>
@@ -998,8 +1083,11 @@
       <c r="F26" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>75</v>
       </c>
@@ -1018,8 +1106,11 @@
       <c r="F27" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G27" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>77</v>
       </c>
@@ -1038,8 +1129,11 @@
       <c r="F28" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G28" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>81</v>
       </c>
@@ -1058,8 +1152,11 @@
       <c r="F29" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G29" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>84</v>
       </c>
@@ -1078,8 +1175,11 @@
       <c r="F30" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>92</v>
       </c>
@@ -1098,8 +1198,11 @@
       <c r="F31" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G31" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>54</v>
       </c>
@@ -1118,8 +1221,11 @@
       <c r="F32" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>59</v>
       </c>
@@ -1138,8 +1244,11 @@
       <c r="F33" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G33" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>63</v>
       </c>
@@ -1158,8 +1267,11 @@
       <c r="F34" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G34" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>69</v>
       </c>
@@ -1178,8 +1290,11 @@
       <c r="F35" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G35" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>71</v>
       </c>
@@ -1198,8 +1313,11 @@
       <c r="F36" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>74</v>
       </c>
@@ -1218,8 +1336,11 @@
       <c r="F37" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>76</v>
       </c>
@@ -1238,8 +1359,11 @@
       <c r="F38" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G38" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>80</v>
       </c>
@@ -1258,8 +1382,11 @@
       <c r="F39" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G39" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>83</v>
       </c>
@@ -1278,8 +1405,11 @@
       <c r="F40" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>91</v>
       </c>
@@ -1297,6 +1427,9 @@
       </c>
       <c r="F41" t="s">
         <v>17</v>
+      </c>
+      <c r="G41" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated mortality and logger files
</commit_message>
<xml_diff>
--- a/data/metadata/experiment_metadata.xlsx
+++ b/data/metadata/experiment_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashuffmyer/MyProjects/oysters/manchester-hardening/data/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B5F8E3-CBAD-7847-A6C6-3094C615985C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6694D14A-A315-764E-92EF-399B333B7CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50220" yWindow="-1100" windowWidth="14060" windowHeight="17600" xr2:uid="{910C5C9C-1199-2F4F-A6BD-E003E55895D4}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{910C5C9C-1199-2F4F-A6BD-E003E55895D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="26">
   <si>
     <t>tank</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>20260528_subsample_tag</t>
   </si>
 </sst>
 </file>
@@ -482,14 +485,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026AE326-2012-A844-AB6A-692D667495E5}">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -511,62 +515,71 @@
       <c r="G1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C2">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+      <c r="H2">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C3">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C4">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -580,77 +593,83 @@
       <c r="G4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C5">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="s">
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G5" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
         <v>10</v>
       </c>
-      <c r="C7">
-        <v>14</v>
-      </c>
       <c r="D7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E7" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>79</v>
       </c>
@@ -673,78 +692,78 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C9">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>18</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
         <v>16</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>2</v>
-      </c>
-      <c r="F9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>87</v>
-      </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10">
-        <v>14</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>2</v>
-      </c>
-      <c r="F10" t="s">
-        <v>19</v>
-      </c>
       <c r="G10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>90</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C11">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -753,27 +772,27 @@
         <v>18</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" t="s">
         <v>2</v>
       </c>
       <c r="F12" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13">
         <v>18</v>
-      </c>
-      <c r="G12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>57</v>
-      </c>
-      <c r="B13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13">
-        <v>45</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -785,87 +804,96 @@
         <v>18</v>
       </c>
       <c r="G13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14">
+        <v>20</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>74</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15">
+        <v>20</v>
+      </c>
+      <c r="D15">
+        <v>4</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>62</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16">
+        <v>20</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>2</v>
+      </c>
+      <c r="F16" t="s">
         <v>19</v>
       </c>
-      <c r="D14">
-        <v>2</v>
-      </c>
-      <c r="E14" t="s">
-        <v>2</v>
-      </c>
-      <c r="F14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" t="s">
+      <c r="G16" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>64</v>
-      </c>
-      <c r="B15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15">
-        <v>17</v>
-      </c>
-      <c r="D15">
-        <v>2</v>
-      </c>
-      <c r="E15" t="s">
-        <v>2</v>
-      </c>
-      <c r="F15" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>67</v>
-      </c>
-      <c r="B16" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16">
-        <v>28</v>
-      </c>
-      <c r="D16">
-        <v>2</v>
-      </c>
-      <c r="E16" t="s">
-        <v>2</v>
-      </c>
-      <c r="F16" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H16">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C17">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D17">
         <v>2</v>
@@ -877,58 +905,61 @@
         <v>18</v>
       </c>
       <c r="G17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+      <c r="H17">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C18">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G18" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C19">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="D19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G19" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s">
         <v>13</v>
@@ -937,27 +968,27 @@
         <v>16</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="s">
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G20" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C21">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D21">
         <v>2</v>
@@ -972,15 +1003,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C22">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -995,84 +1026,84 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="B23" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C23">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="D23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E23" t="s">
         <v>3</v>
       </c>
       <c r="F23" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G23" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C24">
         <v>14</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="B25" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C25">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E25" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C26">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D26">
         <v>3</v>
@@ -1084,87 +1115,99 @@
         <v>16</v>
       </c>
       <c r="G26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+      <c r="H26">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="B27" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C27">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E27" t="s">
         <v>3</v>
       </c>
       <c r="F27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G27" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+      <c r="H27">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C28">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D28">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G28" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+      <c r="H28">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="B29" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C29">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G29" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H29">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="B30" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C30">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D30">
         <v>3</v>
@@ -1179,99 +1222,102 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="B31" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C31">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" t="s">
         <v>3</v>
       </c>
       <c r="F31" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G31" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B32" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C32">
+        <v>17</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32" t="s">
+        <v>2</v>
+      </c>
+      <c r="F32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>64</v>
+      </c>
+      <c r="B33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33">
+        <v>17</v>
+      </c>
+      <c r="D33">
+        <v>2</v>
+      </c>
+      <c r="E33" t="s">
+        <v>2</v>
+      </c>
+      <c r="F33" t="s">
         <v>18</v>
-      </c>
-      <c r="D32">
-        <v>4</v>
-      </c>
-      <c r="E32" t="s">
-        <v>3</v>
-      </c>
-      <c r="F32" t="s">
-        <v>17</v>
-      </c>
-      <c r="G32" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33">
-        <v>59</v>
-      </c>
-      <c r="B33" t="s">
-        <v>7</v>
-      </c>
-      <c r="C33">
-        <v>45</v>
-      </c>
-      <c r="D33">
-        <v>4</v>
-      </c>
-      <c r="E33" t="s">
-        <v>3</v>
-      </c>
-      <c r="F33" t="s">
-        <v>17</v>
       </c>
       <c r="G33" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B34" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C34">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="D34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E34" t="s">
         <v>3</v>
       </c>
       <c r="F34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G34" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+      <c r="H34">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>69</v>
       </c>
@@ -1293,85 +1339,94 @@
       <c r="G35" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H35">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36">
+        <v>65</v>
+      </c>
+      <c r="B36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36">
+        <v>28</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36" t="s">
+        <v>2</v>
+      </c>
+      <c r="F36" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" t="s">
+        <v>24</v>
+      </c>
+      <c r="H36">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>67</v>
+      </c>
+      <c r="B37" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37">
+        <v>28</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>2</v>
+      </c>
+      <c r="F37" t="s">
+        <v>18</v>
+      </c>
+      <c r="G37" t="s">
+        <v>24</v>
+      </c>
+      <c r="H37">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>66</v>
+      </c>
+      <c r="B38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38">
+        <v>14</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39">
         <v>71</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B39" t="s">
         <v>10</v>
       </c>
-      <c r="C36">
+      <c r="C39">
         <v>14</v>
-      </c>
-      <c r="D36">
-        <v>4</v>
-      </c>
-      <c r="E36" t="s">
-        <v>3</v>
-      </c>
-      <c r="F36" t="s">
-        <v>17</v>
-      </c>
-      <c r="G36" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37">
-        <v>74</v>
-      </c>
-      <c r="B37" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37">
-        <v>20</v>
-      </c>
-      <c r="D37">
-        <v>4</v>
-      </c>
-      <c r="E37" t="s">
-        <v>3</v>
-      </c>
-      <c r="F37" t="s">
-        <v>17</v>
-      </c>
-      <c r="G37" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38">
-        <v>76</v>
-      </c>
-      <c r="B38" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38">
-        <v>10</v>
-      </c>
-      <c r="D38">
-        <v>4</v>
-      </c>
-      <c r="E38" t="s">
-        <v>3</v>
-      </c>
-      <c r="F38" t="s">
-        <v>17</v>
-      </c>
-      <c r="G38" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39">
-        <v>80</v>
-      </c>
-      <c r="B39" t="s">
-        <v>14</v>
-      </c>
-      <c r="C39">
-        <v>38</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -1383,59 +1438,59 @@
         <v>17</v>
       </c>
       <c r="G39" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="B40" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C40">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E40" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G40" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C41">
         <v>14</v>
       </c>
       <c r="D41">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E41" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F41" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G41" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F41">
-    <sortCondition ref="D2:D41"/>
-    <sortCondition ref="A2:A41"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G41">
+    <sortCondition ref="B2:B41"/>
+    <sortCondition ref="E2:E41"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>